<commit_message>
Addded API Doc file
</commit_message>
<xml_diff>
--- a/Document/Api Document.xlsx
+++ b/Document/Api Document.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prathamesh\Project\ORVÉA\Document\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAD18A0-350B-4721-A422-0E28E473ABB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Patient Service" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,15 +24,175 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>/api/v1/patients</t>
+  </si>
+  <si>
+    <t>PATIENT_CREATE</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/duplicate-check</t>
+  </si>
+  <si>
+    <t>PATIENT_CREATE or PATIENT_READ</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/search?phone=&amp;name=&amp;uhid=</t>
+  </si>
+  <si>
+    <t>PATIENT_READ</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/me</t>
+  </si>
+  <si>
+    <t>role PATIENT</t>
+  </si>
+  <si>
+    <t>GET/PUT/DELETE</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/{id}</t>
+  </si>
+  <si>
+    <t>READ / UPDATE / DELETE</t>
+  </si>
+  <si>
+    <t>POST/GET</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/{id}/cases</t>
+  </si>
+  <si>
+    <t>TREATMENT_CREATE / READ</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PUT, PATCH </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, POST </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/sessions/complete</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, DELETE</t>
+    </r>
+  </si>
+  <si>
+    <t>.../cases/{caseId}</t>
+  </si>
+  <si>
+    <t>TREATMENT_UPDATE</t>
+  </si>
+  <si>
+    <t>POST/DELETE</t>
+  </si>
+  <si>
+    <t>.../cases/{caseId}/conditions</t>
+  </si>
+  <si>
+    <t>CRUD</t>
+  </si>
+  <si>
+    <t>/api/v1/patients/{id}/care-team</t>
+  </si>
+  <si>
+    <t>PATIENT_UPDATE / READ</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">POST/GET, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/check</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/withdraw</t>
+    </r>
+  </si>
+  <si>
+    <t>/api/v1/patients/{id}/consents</t>
+  </si>
+  <si>
+    <t>/api/v1/conditions</t>
+  </si>
+  <si>
+    <t>SETTINGS_MANAGE (write)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,8 +215,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +503,138 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="35.33203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="47.21875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28.8">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>